<commit_message>
added a .0 to a major version number.
</commit_message>
<xml_diff>
--- a/system_design/Georgetown/V0.5.2/bill_of_materials.xlsx
+++ b/system_design/Georgetown/V0.5.2/bill_of_materials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailsc-my.sharepoint.com/personal/asifuzzaman_sc_edu/Documents/Github Repos/UAV-Deployable-Stage-Height-Sensor/system_design/Georgetown/V0.5.2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adowney2\Documents\GitHub\SWaP-Constrained-UAV-deployable-Water-Level-Sensor\system_design\Georgetown\V0.5.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="13_ncr:1_{92FC9251-22EE-4CB6-81B0-D0434CABC585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A22FF58F-C98B-49F2-8610-E9AF52551917}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADAA0EB-7F46-452A-86E2-E40C43A33CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-16320" yWindow="-6540" windowWidth="16440" windowHeight="28320" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -917,23 +917,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="89.90625" customWidth="1"/>
-    <col min="3" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.54296875" customWidth="1"/>
-    <col min="5" max="5" width="13.08984375" customWidth="1"/>
-    <col min="6" max="6" width="9.1796875" customWidth="1"/>
-    <col min="7" max="7" width="69.453125" customWidth="1"/>
+    <col min="1" max="1" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="89.85546875" customWidth="1"/>
+    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" customWidth="1"/>
+    <col min="7" max="7" width="69.42578125" customWidth="1"/>
     <col min="8" max="8" width="76" customWidth="1"/>
-    <col min="9" max="9" width="83.54296875" customWidth="1"/>
-    <col min="10" max="10" width="62.54296875" customWidth="1"/>
-    <col min="11" max="11" width="55.81640625" customWidth="1"/>
+    <col min="9" max="9" width="83.5703125" customWidth="1"/>
+    <col min="10" max="10" width="62.5703125" customWidth="1"/>
+    <col min="11" max="11" width="55.85546875" customWidth="1"/>
     <col min="12" max="12" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>117</v>
       </c>
@@ -971,7 +971,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>123</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>122</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>109</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>149</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
@@ -1226,7 +1226,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>111</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>145</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>150</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>112</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>119</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>141</v>
       </c>
@@ -1445,7 +1445,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="19" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>102</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>103</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>138</v>
       </c>
@@ -1523,7 +1523,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>104</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>105</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>100</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>144</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>106</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>44</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>13</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>114</v>
       </c>
@@ -1739,7 +1739,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>131</v>
       </c>
@@ -1763,7 +1763,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>134</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>39</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="2" t="s">
         <v>129</v>
       </c>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="G33" s="1"/>
     </row>
-    <row r="34" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="2" t="s">
         <v>130</v>
       </c>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="G34" s="1"/>
     </row>
-    <row r="35" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="2" t="s">
         <v>127</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
         <v>128</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>90</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="38" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>93</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E39" s="4" t="s">
         <v>14</v>
       </c>

</xml_diff>